<commit_message>
ACTUALIZAR DATOS: Subir archivos Excel con información actualizada (Lista Maestra, evaluadores, etc.)
</commit_message>
<xml_diff>
--- a/data/BALANCE DE CARGAS DE TRABAJO_JONATHAN MEDINA.xlsx
+++ b/data/BALANCE DE CARGAS DE TRABAJO_JONATHAN MEDINA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmedina\PyCharmMiscProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAC9C582-6ECF-4B41-8EB3-D9339DD6942F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394C6DC2-687F-4E25-83F0-6971B4583AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MUESTREO" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="CONTENIDO DE TRABAJO" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lista Maestra'!$C$5:$H$190</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lista Maestra'!$C$5:$H$209</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2589" uniqueCount="573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2675" uniqueCount="636">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -787,6 +787,21 @@
     <t>culminé parcialmente tarea 13, pendiente que aprueben y ahi continuo la tarea</t>
   </si>
   <si>
+    <t>ANALISTA CARTERA</t>
+  </si>
+  <si>
+    <t>NICOLE NOBOA</t>
+  </si>
+  <si>
+    <t>05/01/2026</t>
+  </si>
+  <si>
+    <t>16:04:29</t>
+  </si>
+  <si>
+    <t>16:23:33</t>
+  </si>
+  <si>
     <t>REUNIONES</t>
   </si>
   <si>
@@ -1531,6 +1546,9 @@
     <t>Se ingresa a las paginas web de la navieras asigandas y se coloca toda la informacion que van a llevar los contenedores de manera correcta , se ingresa las proformas dentro plazos documentales que cada naviera.</t>
   </si>
   <si>
+    <t>PROFORMAS</t>
+  </si>
+  <si>
     <t>Corregir la informacion que nos envia la naviera de los BLS finales, tomando la informacion de los cierres de contenedores semanales (FTL)</t>
   </si>
   <si>
@@ -1564,10 +1582,16 @@
     <t xml:space="preserve">Ingresamos la informacion en la pagina de la naviera ( Booking - Contenedor) donde colocamos el peso de cada contendor para asi confirmar que los embarque no presenten problemas en cuanto al peso de la nave. </t>
   </si>
   <si>
+    <t>VERIFICACIÓN</t>
+  </si>
+  <si>
     <t xml:space="preserve">DECLARACION DE CARTAR DE TEMPERATURA  NAVIERAS ASIGNADAS </t>
   </si>
   <si>
     <t xml:space="preserve">Se ingresa a las paginas web de la navieras o se realiza plantillas en Excel donde se coloca toda la informacion y las especificaciones de las temperatura que solicita cada cliente para cada producto.  </t>
+  </si>
+  <si>
+    <t>DECLARACIONES</t>
   </si>
   <si>
     <t>LIBERACION DE BLS SWB (Contenedores) POR PAGOS PENDIENTES
@@ -1577,9 +1601,15 @@
     <t>Se solicita a la naviera liberacion por correo despues de cancelar los valores a pagar por las exportaciones y asi solicitar el envio de los BLS (SWB) despues que las naves zarparan y se exportaran todos los contenedores.</t>
   </si>
   <si>
+    <t>GESTIÓN NAVIERA</t>
+  </si>
+  <si>
     <t>Una vez regularizada las DAES de las navieras asignadas se recopila la siguentes informacion: DAE regularizada, factura, BLS , capture del estado regularizada en el ECUAPASS , se realiza  1 PDF con esos 4 documentos y se los coloca en la red.</t>
   </si>
   <si>
+    <t>DIGITALIZACIONES</t>
+  </si>
+  <si>
     <t>REDUCION DE DAES                                                                                    ( CMA -  KING OCEAN   ONE -  SEABOARD )</t>
   </si>
   <si>
@@ -1610,6 +1640,9 @@
     <t>SOPORTE EN DOCUMENTOS FITOSANITARIOS</t>
   </si>
   <si>
+    <t>SOPORTE</t>
+  </si>
+  <si>
     <t>Reportar siniestros property</t>
   </si>
   <si>
@@ -1745,6 +1778,185 @@
     <t>Reunión con deparamentos contiguos tales como COMEX.</t>
   </si>
   <si>
+    <t>Actualizar y publicar del portafolio</t>
+  </si>
+  <si>
+    <t>Registrar las facturas enviadas por el departamento comercial, junto con las ventas proformadas y la mercadería en tránsito.
+Validar que los valores facturados coincidan con los registrados en SAP.
+Actualizar la proyección de ventas correspondientes a la semana en curso.
+Revisar los pagos recibidos y las notas de crédito emitidas.
+Ejecutar la información mediante el programa R para su procesamiento y actualización de resultados en Power BI.</t>
+  </si>
+  <si>
+    <t>ELABORACIÓN DE PORTAFOLIO</t>
+  </si>
+  <si>
+    <t>Actualizar fondeo Lineal (historico)</t>
+  </si>
+  <si>
+    <t>Actializar las ventas semanales (SAP) y las notas de crédito descontadas.
+Detallar el saldo semanal de la liquidez pendiente correspondiente a la cartera total.</t>
+  </si>
+  <si>
+    <t>ACTUALIZACIÓN DE FLUJO HISTÓRICO</t>
+  </si>
+  <si>
+    <t>Realizar del fondeo (ingresos)</t>
+  </si>
+  <si>
+    <t>Registrar las ventas de la semana en curso (Expocredit, Liquidez, Standard y venta directa).
+Planificar las reservas disponibles de las operaciones de factoring, notas de créditos, descuentos y cobros directos.</t>
+  </si>
+  <si>
+    <t>ELABORACIÓN DE FONDEO</t>
+  </si>
+  <si>
+    <t>Documentar y ejecutar ventas factoring</t>
+  </si>
+  <si>
+    <t>Realizar los anexos y detalles de las ventas semanales (Expocredit, Liquidez Plus)</t>
+  </si>
+  <si>
+    <t>DOCUMENTACIÓN FACTORING</t>
+  </si>
+  <si>
+    <t>Actualizar reservas operaciones factoring (Expocredit)</t>
+  </si>
+  <si>
+    <t>Descargar los archivos PDF de los collections liberados desde la plataforma de Expocredit y actualizar la información correspondiente en el archivo Excel de control.</t>
+  </si>
+  <si>
+    <t>ACTUALIZACIÓN DE RESERVAS FACTORING</t>
+  </si>
+  <si>
+    <t>Alimentar archivo de gasto financiero</t>
+  </si>
+  <si>
+    <t>Actualizar las ventas proformadas, categorizadas en plátano y banano.
+Detallar la semana de liquidación de las reservas recibidas.</t>
+  </si>
+  <si>
+    <t>ACTUALIZACIÓN DE GASTOS FINANCIEROS</t>
+  </si>
+  <si>
+    <t>Coordinar y dirigir comité de cartera</t>
+  </si>
+  <si>
+    <t>Exponer las etapas de gestión, comportamiento de pagos, revisión de detalles de gasto financiero y revisión de cobertura de crédito
+Desarrolar los casos de cartera que se presenten.</t>
+  </si>
+  <si>
+    <t>COMITÉ DE CARTERA</t>
+  </si>
+  <si>
+    <t>Realizar anexo de gastos financieros y CXC</t>
+  </si>
+  <si>
+    <t>Actualizar los reportes de cierre de mes de los intereses y de los saldos en las cuentas correspondientes (SAP).</t>
+  </si>
+  <si>
+    <t>ELABORACIÓN DE ANEXOS</t>
+  </si>
+  <si>
+    <t>Enviar analisis semanal</t>
+  </si>
+  <si>
+    <t>Enviar por correo el PDF del análisis semanal Spurrier e imprimir dos ejemplares para el Gerente Financiero y Sub Gerente Financiero.</t>
+  </si>
+  <si>
+    <t>ANÁLISIS SPURRIER</t>
+  </si>
+  <si>
+    <t>Enviar estados de cuenta</t>
+  </si>
+  <si>
+    <t>Enviar los estados de cuenta a los clientes que se encuentren en las etapas de gestión del 1 al 4.</t>
+  </si>
+  <si>
+    <t>ESTADOS DE CUENTA CLIENTES</t>
+  </si>
+  <si>
+    <t>Descargar de estados de cuenta</t>
+  </si>
+  <si>
+    <t>Descargar los estados de cuenta de las entidades bancarias.</t>
+  </si>
+  <si>
+    <t>ESTADOS DE CUENTA BANCARIOS</t>
+  </si>
+  <si>
+    <t>Registrar de créditos</t>
+  </si>
+  <si>
+    <t>Registrar los créditos categorizados en: ventas factoring, reservas, cobros directos e ingresos varios.</t>
+  </si>
+  <si>
+    <t>REGISTRO DE CRÉDITOS BANCARIOS</t>
+  </si>
+  <si>
+    <t>Renovar cupos de seguro de crédito</t>
+  </si>
+  <si>
+    <t>Enviar al broker la proyección de ventas anual del próximo año y la necesidad de cupo por cliente.</t>
+  </si>
+  <si>
+    <t>GESTIÓN CUPOS DE CRÉDITO</t>
+  </si>
+  <si>
+    <t>Enviar detalles de aplicación de cobros</t>
+  </si>
+  <si>
+    <t>Enviar los detalles de cobros y la confirmación a Expocredit.</t>
+  </si>
+  <si>
+    <t>DETALLES DE PAGO</t>
+  </si>
+  <si>
+    <t>Compensar anticipos clientes</t>
+  </si>
+  <si>
+    <t>Revisar y reconciliar los anticipos pendientes de aplicación al cierre del mes.</t>
+  </si>
+  <si>
+    <t>COMPENSACIÓN DE ANTICIPOS</t>
+  </si>
+  <si>
+    <t>Realizar conciliaciones exportadoras</t>
+  </si>
+  <si>
+    <t>Reconciliar los anticipos y facturas entre las empresas exportadoras</t>
+  </si>
+  <si>
+    <t>CONCILIACIÓN EXPORTACIÓN</t>
+  </si>
+  <si>
+    <t>Envío de detalle y emisión de notas de créditos</t>
+  </si>
+  <si>
+    <t>identificar y detallar las notas de créditos descontada.</t>
+  </si>
+  <si>
+    <t>NOTAS DE CRÉDITO</t>
+  </si>
+  <si>
+    <t>Asignación de números de pedidos para la mercadería en tránsito</t>
+  </si>
+  <si>
+    <t>Designar el número de PO correspondiente a la semana en tránsito de la carga de COSCTO, según el detalle proporcionado por el departamento de Comex.</t>
+  </si>
+  <si>
+    <t>ASIGNACIÓN POs</t>
+  </si>
+  <si>
+    <t>Reporte de siniestro Coface</t>
+  </si>
+  <si>
+    <t>Reportar y documentar el caso en la plataforma coface.</t>
+  </si>
+  <si>
+    <t>SINIESTRO SEGURO</t>
+  </si>
+  <si>
     <t>EXP GROUP LLC</t>
   </si>
   <si>
@@ -1844,22 +2056,7 @@
     <t>0.38.26</t>
   </si>
   <si>
-    <t>PROFORMAS</t>
-  </si>
-  <si>
-    <t>VERIFICACIÓN</t>
-  </si>
-  <si>
-    <t>DECLARACIONES</t>
-  </si>
-  <si>
-    <t>GESTIÓN NAVIERA</t>
-  </si>
-  <si>
-    <t>DIGITALIZACIONES</t>
-  </si>
-  <si>
-    <t>SOPORTE</t>
+    <t>DEFINIR PROCESOS Y CRITERIOS INGENIERILES</t>
   </si>
 </sst>
 </file>
@@ -2193,7 +2390,7 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment wrapText="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -2235,7 +2432,7 @@
         <family val="2"/>
       </font>
       <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
       <font>
@@ -2757,8 +2954,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MUESTREO_LABORAL_A2" displayName="MUESTREO_LABORAL_A2" ref="B3:R331" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="B3:R331" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MUESTREO_LABORAL_A2" displayName="MUESTREO_LABORAL_A2" ref="B3:R328" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+  <autoFilter ref="B3:R328" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="EMPRESA" dataDxfId="20"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="DEPARTAMENTO" dataDxfId="19"/>
@@ -3105,7 +3302,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:S331"/>
+  <dimension ref="B3:S328"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -3578,9 +3775,9 @@
         <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,3,0),"")</f>
         <v>DEFINICIÓN</v>
       </c>
-      <c r="K12" s="31">
-        <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,2,0),"")</f>
-        <v>0</v>
+      <c r="K12" s="31" t="str">
+        <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,2,0),"")</f>
+        <v>DEFINIR PROCESOS Y CRITERIOS INGENIERILES</v>
       </c>
       <c r="L12" s="8" t="s">
         <v>35</v>
@@ -3958,9 +4155,9 @@
         <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,3,0),"")</f>
         <v>DEFINICIÓN</v>
       </c>
-      <c r="K20" s="31">
-        <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,2,0),"")</f>
-        <v>0</v>
+      <c r="K20" s="31" t="str">
+        <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,2,0),"")</f>
+        <v>DEFINIR PROCESOS Y CRITERIOS INGENIERILES</v>
       </c>
       <c r="L20" s="17" t="s">
         <v>35</v>
@@ -5541,7 +5738,7 @@
       </c>
       <c r="R54" s="12"/>
     </row>
-    <row r="55" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="2" t="s">
         <v>64</v>
       </c>
@@ -5688,7 +5885,7 @@
       <c r="Q57" s="12"/>
       <c r="R57" s="12"/>
     </row>
-    <row r="58" spans="2:18" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:18" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="2" t="s">
         <v>64</v>
       </c>
@@ -6965,9 +7162,9 @@
         <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,3,0),"")</f>
         <v>DEFINICIÓN</v>
       </c>
-      <c r="K84" s="31">
-        <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,2,0),"")</f>
-        <v>0</v>
+      <c r="K84" s="31" t="str">
+        <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,2,0),"")</f>
+        <v>DEFINIR PROCESOS Y CRITERIOS INGENIERILES</v>
       </c>
       <c r="L84" s="8" t="s">
         <v>35</v>
@@ -6986,7 +7183,7 @@
       <c r="Q84" s="12"/>
       <c r="R84" s="12"/>
     </row>
-    <row r="85" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B85" s="8" t="s">
         <v>17</v>
       </c>
@@ -7032,7 +7229,7 @@
       <c r="Q85" s="12"/>
       <c r="R85" s="12"/>
     </row>
-    <row r="86" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B86" s="8" t="s">
         <v>17</v>
       </c>
@@ -7080,7 +7277,7 @@
       </c>
       <c r="R86" s="12"/>
     </row>
-    <row r="87" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B87" s="8" t="s">
         <v>17</v>
       </c>
@@ -7126,7 +7323,7 @@
       <c r="Q87" s="12"/>
       <c r="R87" s="12"/>
     </row>
-    <row r="88" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B88" s="8" t="s">
         <v>17</v>
       </c>
@@ -7172,7 +7369,7 @@
       <c r="Q88" s="12"/>
       <c r="R88" s="12"/>
     </row>
-    <row r="89" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B89" s="8" t="s">
         <v>17</v>
       </c>
@@ -7218,7 +7415,7 @@
       <c r="Q89" s="12"/>
       <c r="R89" s="12"/>
     </row>
-    <row r="90" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B90" s="8" t="s">
         <v>17</v>
       </c>
@@ -7454,7 +7651,7 @@
       </c>
       <c r="R94" s="12"/>
     </row>
-    <row r="95" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B95" s="8" t="s">
         <v>17</v>
       </c>
@@ -7500,7 +7697,7 @@
       <c r="Q95" s="12"/>
       <c r="R95" s="12"/>
     </row>
-    <row r="96" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B96" s="8" t="s">
         <v>17</v>
       </c>
@@ -7546,7 +7743,7 @@
       <c r="Q96" s="12"/>
       <c r="R96" s="12"/>
     </row>
-    <row r="97" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B97" s="8" t="s">
         <v>17</v>
       </c>
@@ -7592,7 +7789,7 @@
       <c r="Q97" s="12"/>
       <c r="R97" s="12"/>
     </row>
-    <row r="98" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B98" s="8" t="s">
         <v>17</v>
       </c>
@@ -7638,7 +7835,7 @@
       <c r="Q98" s="12"/>
       <c r="R98" s="12"/>
     </row>
-    <row r="99" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B99" s="8" t="s">
         <v>17</v>
       </c>
@@ -7730,7 +7927,7 @@
       <c r="Q100" s="12"/>
       <c r="R100" s="12"/>
     </row>
-    <row r="101" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B101" s="8" t="s">
         <v>17</v>
       </c>
@@ -7776,7 +7973,7 @@
       <c r="Q101" s="12"/>
       <c r="R101" s="12"/>
     </row>
-    <row r="102" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B102" s="8" t="s">
         <v>17</v>
       </c>
@@ -7868,7 +8065,7 @@
       <c r="Q103" s="12"/>
       <c r="R103" s="12"/>
     </row>
-    <row r="104" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B104" s="8" t="s">
         <v>17</v>
       </c>
@@ -7960,7 +8157,7 @@
       <c r="Q105" s="12"/>
       <c r="R105" s="12"/>
     </row>
-    <row r="106" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B106" s="8" t="s">
         <v>17</v>
       </c>
@@ -8052,7 +8249,7 @@
       <c r="Q107" s="12"/>
       <c r="R107" s="12"/>
     </row>
-    <row r="108" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B108" s="8" t="s">
         <v>17</v>
       </c>
@@ -8098,7 +8295,7 @@
       <c r="Q108" s="12"/>
       <c r="R108" s="12"/>
     </row>
-    <row r="109" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B109" s="8" t="s">
         <v>17</v>
       </c>
@@ -8144,7 +8341,7 @@
       <c r="Q109" s="12"/>
       <c r="R109" s="12"/>
     </row>
-    <row r="110" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B110" s="8" t="s">
         <v>17</v>
       </c>
@@ -8190,7 +8387,7 @@
       <c r="Q110" s="12"/>
       <c r="R110" s="12"/>
     </row>
-    <row r="111" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B111" s="8" t="s">
         <v>17</v>
       </c>
@@ -8374,7 +8571,7 @@
       <c r="Q114" s="12"/>
       <c r="R114" s="12"/>
     </row>
-    <row r="115" spans="2:18" ht="69" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:18" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B115" s="8" t="s">
         <v>17</v>
       </c>
@@ -8420,7 +8617,7 @@
       <c r="Q115" s="12"/>
       <c r="R115" s="12"/>
     </row>
-    <row r="116" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B116" s="8" t="s">
         <v>17</v>
       </c>
@@ -8466,7 +8663,7 @@
       <c r="Q116" s="12"/>
       <c r="R116" s="12"/>
     </row>
-    <row r="117" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B117" s="8" t="s">
         <v>17</v>
       </c>
@@ -8604,7 +8801,7 @@
       <c r="Q119" s="12"/>
       <c r="R119" s="12"/>
     </row>
-    <row r="120" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B120" s="8" t="s">
         <v>17</v>
       </c>
@@ -8650,7 +8847,7 @@
       <c r="Q120" s="12"/>
       <c r="R120" s="12"/>
     </row>
-    <row r="121" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B121" s="8" t="s">
         <v>17</v>
       </c>
@@ -8742,7 +8939,7 @@
       <c r="Q122" s="12"/>
       <c r="R122" s="12"/>
     </row>
-    <row r="123" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B123" s="8" t="s">
         <v>17</v>
       </c>
@@ -8788,7 +8985,7 @@
       <c r="Q123" s="12"/>
       <c r="R123" s="12"/>
     </row>
-    <row r="124" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B124" s="8" t="s">
         <v>17</v>
       </c>
@@ -8880,7 +9077,7 @@
       <c r="Q125" s="12"/>
       <c r="R125" s="12"/>
     </row>
-    <row r="126" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B126" s="8" t="s">
         <v>17</v>
       </c>
@@ -8972,7 +9169,7 @@
       <c r="Q127" s="12"/>
       <c r="R127" s="12"/>
     </row>
-    <row r="128" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B128" s="8" t="s">
         <v>17</v>
       </c>
@@ -9018,7 +9215,7 @@
       <c r="Q128" s="12"/>
       <c r="R128" s="12"/>
     </row>
-    <row r="129" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B129" s="8" t="s">
         <v>17</v>
       </c>
@@ -9064,7 +9261,7 @@
       <c r="Q129" s="12"/>
       <c r="R129" s="12"/>
     </row>
-    <row r="130" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B130" s="8" t="s">
         <v>17</v>
       </c>
@@ -9156,7 +9353,7 @@
       <c r="Q131" s="12"/>
       <c r="R131" s="12"/>
     </row>
-    <row r="132" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B132" s="8" t="s">
         <v>17</v>
       </c>
@@ -9248,7 +9445,7 @@
       <c r="Q133" s="12"/>
       <c r="R133" s="12"/>
     </row>
-    <row r="134" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B134" s="8" t="s">
         <v>17</v>
       </c>
@@ -9294,7 +9491,7 @@
       <c r="Q134" s="12"/>
       <c r="R134" s="12"/>
     </row>
-    <row r="135" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B135" s="8" t="s">
         <v>17</v>
       </c>
@@ -9340,7 +9537,7 @@
       <c r="Q135" s="12"/>
       <c r="R135" s="12"/>
     </row>
-    <row r="136" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B136" s="8" t="s">
         <v>17</v>
       </c>
@@ -9432,7 +9629,7 @@
       <c r="Q137" s="12"/>
       <c r="R137" s="12"/>
     </row>
-    <row r="138" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B138" s="8" t="s">
         <v>17</v>
       </c>
@@ -9478,7 +9675,7 @@
       <c r="Q138" s="12"/>
       <c r="R138" s="12"/>
     </row>
-    <row r="139" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B139" s="8" t="s">
         <v>17</v>
       </c>
@@ -9524,7 +9721,7 @@
       <c r="Q139" s="12"/>
       <c r="R139" s="12"/>
     </row>
-    <row r="140" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B140" s="8" t="s">
         <v>17</v>
       </c>
@@ -9570,7 +9767,7 @@
       <c r="Q140" s="12"/>
       <c r="R140" s="12"/>
     </row>
-    <row r="141" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B141" s="8" t="s">
         <v>17</v>
       </c>
@@ -9616,7 +9813,7 @@
       <c r="Q141" s="12"/>
       <c r="R141" s="12"/>
     </row>
-    <row r="142" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B142" s="8" t="s">
         <v>17</v>
       </c>
@@ -9662,7 +9859,7 @@
       <c r="Q142" s="12"/>
       <c r="R142" s="12"/>
     </row>
-    <row r="143" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B143" s="8" t="s">
         <v>17</v>
       </c>
@@ -9708,7 +9905,7 @@
       <c r="Q143" s="12"/>
       <c r="R143" s="12"/>
     </row>
-    <row r="144" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B144" s="8" t="s">
         <v>17</v>
       </c>
@@ -9754,7 +9951,7 @@
       <c r="Q144" s="12"/>
       <c r="R144" s="12"/>
     </row>
-    <row r="145" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B145" s="8" t="s">
         <v>17</v>
       </c>
@@ -9800,7 +9997,7 @@
       <c r="Q145" s="12"/>
       <c r="R145" s="12"/>
     </row>
-    <row r="146" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B146" s="8" t="s">
         <v>17</v>
       </c>
@@ -9846,7 +10043,7 @@
       <c r="Q146" s="12"/>
       <c r="R146" s="12"/>
     </row>
-    <row r="147" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B147" s="8" t="s">
         <v>17</v>
       </c>
@@ -9892,7 +10089,7 @@
       <c r="Q147" s="12"/>
       <c r="R147" s="12"/>
     </row>
-    <row r="148" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B148" s="8" t="s">
         <v>17</v>
       </c>
@@ -9938,7 +10135,7 @@
       <c r="Q148" s="12"/>
       <c r="R148" s="12"/>
     </row>
-    <row r="149" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B149" s="8" t="s">
         <v>17</v>
       </c>
@@ -9984,7 +10181,7 @@
       <c r="Q149" s="12"/>
       <c r="R149" s="12"/>
     </row>
-    <row r="150" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B150" s="8" t="s">
         <v>17</v>
       </c>
@@ -10030,7 +10227,7 @@
       <c r="Q150" s="12"/>
       <c r="R150" s="12"/>
     </row>
-    <row r="151" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B151" s="8" t="s">
         <v>17</v>
       </c>
@@ -10076,7 +10273,7 @@
       <c r="Q151" s="12"/>
       <c r="R151" s="12"/>
     </row>
-    <row r="152" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B152" s="8" t="s">
         <v>17</v>
       </c>
@@ -10168,7 +10365,7 @@
       <c r="Q153" s="12"/>
       <c r="R153" s="12"/>
     </row>
-    <row r="154" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B154" s="8" t="s">
         <v>17</v>
       </c>
@@ -10214,7 +10411,7 @@
       <c r="Q154" s="12"/>
       <c r="R154" s="12"/>
     </row>
-    <row r="155" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B155" s="8" t="s">
         <v>17</v>
       </c>
@@ -10260,7 +10457,7 @@
       <c r="Q155" s="12"/>
       <c r="R155" s="12"/>
     </row>
-    <row r="156" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="156" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B156" s="8" t="s">
         <v>17</v>
       </c>
@@ -10306,7 +10503,7 @@
       <c r="Q156" s="12"/>
       <c r="R156" s="12"/>
     </row>
-    <row r="157" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="157" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B157" s="8" t="s">
         <v>17</v>
       </c>
@@ -10398,7 +10595,7 @@
       <c r="Q158" s="12"/>
       <c r="R158" s="12"/>
     </row>
-    <row r="159" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B159" s="8" t="s">
         <v>17</v>
       </c>
@@ -10444,7 +10641,7 @@
       <c r="Q159" s="12"/>
       <c r="R159" s="12"/>
     </row>
-    <row r="160" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B160" s="8" t="s">
         <v>17</v>
       </c>
@@ -10490,7 +10687,7 @@
       <c r="Q160" s="12"/>
       <c r="R160" s="12"/>
     </row>
-    <row r="161" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B161" s="8" t="s">
         <v>17</v>
       </c>
@@ -10536,7 +10733,7 @@
       <c r="Q161" s="12"/>
       <c r="R161" s="12"/>
     </row>
-    <row r="162" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B162" s="8" t="s">
         <v>17</v>
       </c>
@@ -10674,7 +10871,7 @@
       <c r="Q164" s="12"/>
       <c r="R164" s="12"/>
     </row>
-    <row r="165" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B165" s="8" t="s">
         <v>17</v>
       </c>
@@ -10812,7 +11009,7 @@
       <c r="Q167" s="12"/>
       <c r="R167" s="12"/>
     </row>
-    <row r="168" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B168" s="8" t="s">
         <v>17</v>
       </c>
@@ -10858,7 +11055,7 @@
       <c r="Q168" s="12"/>
       <c r="R168" s="12"/>
     </row>
-    <row r="169" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B169" s="8" t="s">
         <v>17</v>
       </c>
@@ -10904,7 +11101,7 @@
       <c r="Q169" s="12"/>
       <c r="R169" s="12"/>
     </row>
-    <row r="170" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B170" s="8" t="s">
         <v>17</v>
       </c>
@@ -10996,7 +11193,7 @@
       <c r="Q171" s="12"/>
       <c r="R171" s="12"/>
     </row>
-    <row r="172" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B172" s="8" t="s">
         <v>17</v>
       </c>
@@ -11042,7 +11239,7 @@
       <c r="Q172" s="12"/>
       <c r="R172" s="12"/>
     </row>
-    <row r="173" spans="2:18" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:18" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B173" s="8" t="s">
         <v>17</v>
       </c>
@@ -11088,7 +11285,7 @@
       <c r="Q173" s="12"/>
       <c r="R173" s="12"/>
     </row>
-    <row r="174" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B174" s="8" t="s">
         <v>17</v>
       </c>
@@ -11134,7 +11331,7 @@
       <c r="Q174" s="12"/>
       <c r="R174" s="12"/>
     </row>
-    <row r="175" spans="2:18" ht="69" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:18" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B175" s="8" t="s">
         <v>17</v>
       </c>
@@ -11226,7 +11423,7 @@
       <c r="Q176" s="12"/>
       <c r="R176" s="12"/>
     </row>
-    <row r="177" spans="2:18" ht="69" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:18" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B177" s="8" t="s">
         <v>17</v>
       </c>
@@ -11318,7 +11515,7 @@
       <c r="Q178" s="12"/>
       <c r="R178" s="12"/>
     </row>
-    <row r="179" spans="2:18" ht="69" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:18" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B179" s="8" t="s">
         <v>17</v>
       </c>
@@ -11364,7 +11561,7 @@
       <c r="Q179" s="12"/>
       <c r="R179" s="12"/>
     </row>
-    <row r="180" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B180" s="8" t="s">
         <v>17</v>
       </c>
@@ -11410,7 +11607,7 @@
       <c r="Q180" s="12"/>
       <c r="R180" s="12"/>
     </row>
-    <row r="181" spans="2:18" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B181" s="8" t="s">
         <v>17</v>
       </c>
@@ -15086,7 +15283,7 @@
       <c r="Q259" s="12"/>
       <c r="R259" s="12"/>
     </row>
-    <row r="260" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="260" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B260" s="2" t="s">
         <v>17</v>
       </c>
@@ -15180,7 +15377,7 @@
       </c>
       <c r="R261" s="12"/>
     </row>
-    <row r="262" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="262" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B262" s="2" t="s">
         <v>17</v>
       </c>
@@ -15226,7 +15423,7 @@
       <c r="Q262" s="12"/>
       <c r="R262" s="12"/>
     </row>
-    <row r="263" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="263" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B263" s="2" t="s">
         <v>17</v>
       </c>
@@ -15272,7 +15469,7 @@
       <c r="Q263" s="12"/>
       <c r="R263" s="12"/>
     </row>
-    <row r="264" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="264" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B264" s="2" t="s">
         <v>17</v>
       </c>
@@ -15828,7 +16025,7 @@
       <c r="Q275" s="12"/>
       <c r="R275" s="12"/>
     </row>
-    <row r="276" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="276" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B276" s="2" t="s">
         <v>17</v>
       </c>
@@ -15920,7 +16117,7 @@
       <c r="Q277" s="12"/>
       <c r="R277" s="12"/>
     </row>
-    <row r="278" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="278" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B278" s="2" t="s">
         <v>17</v>
       </c>
@@ -16058,7 +16255,7 @@
       <c r="Q280" s="12"/>
       <c r="R280" s="12"/>
     </row>
-    <row r="281" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="281" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B281" s="2" t="s">
         <v>17</v>
       </c>
@@ -16104,7 +16301,7 @@
       <c r="Q281" s="12"/>
       <c r="R281" s="12"/>
     </row>
-    <row r="282" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="282" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B282" s="2" t="s">
         <v>17</v>
       </c>
@@ -16152,7 +16349,7 @@
       </c>
       <c r="R282" s="12"/>
     </row>
-    <row r="283" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="283" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B283" s="2" t="s">
         <v>17</v>
       </c>
@@ -16244,7 +16441,7 @@
       <c r="Q284" s="12"/>
       <c r="R284" s="12"/>
     </row>
-    <row r="285" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="285" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B285" s="2" t="s">
         <v>17</v>
       </c>
@@ -16336,7 +16533,7 @@
       <c r="Q286" s="12"/>
       <c r="R286" s="12"/>
     </row>
-    <row r="287" spans="2:18" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="287" spans="2:18" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B287" s="2" t="s">
         <v>17</v>
       </c>
@@ -16383,27 +16580,47 @@
       <c r="R287" s="12"/>
     </row>
     <row r="288" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="D288" s="8"/>
-      <c r="E288" s="8"/>
-      <c r="F288" s="9"/>
+      <c r="B288" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C288" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D288" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="E288" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="F288" s="9" t="s">
+        <v>219</v>
+      </c>
       <c r="G288" s="9"/>
       <c r="H288" s="8"/>
-      <c r="I288" s="8"/>
+      <c r="I288" s="8" t="s">
+        <v>35</v>
+      </c>
       <c r="J288" s="31" t="str">
         <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,3,0),"")</f>
-        <v/>
+        <v>DEFINICIÓN</v>
       </c>
       <c r="K288" s="31" t="str">
         <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="L288" s="8"/>
+        <v>DEFINIR PROCESOS Y CRITERIOS INGENIERILES</v>
+      </c>
+      <c r="L288" s="8" t="s">
+        <v>35</v>
+      </c>
       <c r="M288" s="8"/>
-      <c r="N288" s="10"/>
-      <c r="O288" s="10"/>
-      <c r="P288" s="7" t="str">
-        <f>IF(MUESTREO_LABORAL_A2[[#This Row],[TIEMPO INICIO]]="","",(MUESTREO_LABORAL_A2[[#This Row],[TIEMPO FIN]]-MUESTREO_LABORAL_A2[[#This Row],[TIEMPO INICIO]])*24)</f>
-        <v/>
+      <c r="N288" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="O288" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="P288" s="7">
+        <f>IF(MUESTREO_LABORAL_A2[[#This Row],[TIEMPO INICIO]]="","",(MUESTREO_LABORAL_A2[[#This Row],[TIEMPO FIN]]-MUESTREO_LABORAL_A2[[#This Row],[TIEMPO INICIO]])*24)</f>
+        <v>0.31777777777777594</v>
       </c>
       <c r="Q288" s="12"/>
       <c r="R288" s="12"/>
@@ -17448,86 +17665,8 @@
       <c r="Q328" s="12"/>
       <c r="R328" s="12"/>
     </row>
-    <row r="329" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D329" s="8"/>
-      <c r="E329" s="8"/>
-      <c r="F329" s="9"/>
-      <c r="G329" s="9"/>
-      <c r="H329" s="8"/>
-      <c r="I329" s="8"/>
-      <c r="J329" s="31" t="str">
-        <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,3,0),"")</f>
-        <v/>
-      </c>
-      <c r="K329" s="31" t="str">
-        <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="L329" s="8"/>
-      <c r="M329" s="8"/>
-      <c r="N329" s="10"/>
-      <c r="O329" s="10"/>
-      <c r="P329" s="7" t="str">
-        <f>IF(MUESTREO_LABORAL_A2[[#This Row],[TIEMPO INICIO]]="","",(MUESTREO_LABORAL_A2[[#This Row],[TIEMPO FIN]]-MUESTREO_LABORAL_A2[[#This Row],[TIEMPO INICIO]])*24)</f>
-        <v/>
-      </c>
-      <c r="Q329" s="12"/>
-      <c r="R329" s="12"/>
-    </row>
-    <row r="330" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D330" s="8"/>
-      <c r="E330" s="8"/>
-      <c r="F330" s="9"/>
-      <c r="G330" s="9"/>
-      <c r="H330" s="8"/>
-      <c r="I330" s="8"/>
-      <c r="J330" s="31" t="str">
-        <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,3,0),"")</f>
-        <v/>
-      </c>
-      <c r="K330" s="31" t="str">
-        <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="L330" s="8"/>
-      <c r="M330" s="8"/>
-      <c r="N330" s="10"/>
-      <c r="O330" s="10"/>
-      <c r="P330" s="7" t="str">
-        <f>IF(MUESTREO_LABORAL_A2[[#This Row],[TIEMPO INICIO]]="","",(MUESTREO_LABORAL_A2[[#This Row],[TIEMPO FIN]]-MUESTREO_LABORAL_A2[[#This Row],[TIEMPO INICIO]])*24)</f>
-        <v/>
-      </c>
-      <c r="Q330" s="12"/>
-      <c r="R330" s="12"/>
-    </row>
-    <row r="331" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D331" s="8"/>
-      <c r="E331" s="8"/>
-      <c r="F331" s="9"/>
-      <c r="G331" s="9"/>
-      <c r="H331" s="8"/>
-      <c r="I331" s="8"/>
-      <c r="J331" s="31" t="str">
-        <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,3,0),"")</f>
-        <v/>
-      </c>
-      <c r="K331" s="31" t="str">
-        <f>IFERROR(VLOOKUP(MUESTREO_LABORAL_A2[[#This Row],[ACTIVIDAD]],'Lista Maestra'!$D$6:$F$190,2,0),"")</f>
-        <v/>
-      </c>
-      <c r="L331" s="8"/>
-      <c r="M331" s="8"/>
-      <c r="N331" s="10"/>
-      <c r="O331" s="10"/>
-      <c r="P331" s="7" t="str">
-        <f>IF(MUESTREO_LABORAL_A2[[#This Row],[TIEMPO INICIO]]="","",(MUESTREO_LABORAL_A2[[#This Row],[TIEMPO FIN]]-MUESTREO_LABORAL_A2[[#This Row],[TIEMPO INICIO]])*24)</f>
-        <v/>
-      </c>
-      <c r="Q331" s="12"/>
-      <c r="R331" s="12"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="L4:M331">
+  <conditionalFormatting sqref="L4:M328">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"SIN ACTIVIDAD"</formula>
     </cfRule>
@@ -17535,7 +17674,7 @@
       <formula>"ENC"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M4:M11 M14:M331">
+  <conditionalFormatting sqref="M4:M11 M14:M328">
     <cfRule type="expression" dxfId="1" priority="12">
       <formula>$L4="ENC"</formula>
     </cfRule>
@@ -17566,53 +17705,53 @@
   <sheetData>
     <row r="5" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D5" s="37" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="E5" s="37" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="F5" s="37" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="G5" s="37" t="s">
         <v>8</v>
       </c>
       <c r="H5" s="37" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="I5" s="37" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="6" spans="4:9" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D6" s="24" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="F6" s="29" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="G6" s="45" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="H6" s="45" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="I6" s="45" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D7" s="24" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="F7" s="29" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="G7" s="46"/>
       <c r="H7" s="46"/>
@@ -17621,10 +17760,10 @@
     <row r="8" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D8" s="24"/>
       <c r="E8" s="29" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="F8" s="29" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="G8" s="46"/>
       <c r="H8" s="46"/>
@@ -17633,10 +17772,10 @@
     <row r="9" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D9" s="24"/>
       <c r="E9" s="29" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="G9" s="46"/>
       <c r="H9" s="46"/>
@@ -17648,7 +17787,7 @@
         <v>106</v>
       </c>
       <c r="F10" s="29" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="G10" s="47"/>
       <c r="H10" s="47"/>
@@ -17710,7 +17849,7 @@
         <v>10</v>
       </c>
       <c r="H5" s="21" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="I5" s="13"/>
     </row>
@@ -17722,16 +17861,16 @@
         <v>24</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="F6" s="27" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="G6" s="27" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="H6" s="27" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="I6" s="13"/>
     </row>
@@ -17743,16 +17882,16 @@
         <v>52</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="F7" s="27" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="G7" s="30" t="s">
         <v>30</v>
       </c>
       <c r="H7" s="27" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="I7" s="13"/>
     </row>
@@ -17764,16 +17903,16 @@
         <v>21</v>
       </c>
       <c r="E8" s="27" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="G8" s="27" t="s">
         <v>27</v>
       </c>
       <c r="H8" s="27" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I8" s="13"/>
     </row>
@@ -17782,19 +17921,19 @@
         <v>17</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="F9" s="27" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="G9" s="27" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="H9" s="27" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="I9" s="13"/>
     </row>
@@ -17806,16 +17945,16 @@
         <v>60</v>
       </c>
       <c r="E10" s="27" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="F10" s="27" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="G10" s="27" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="H10" s="27" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="I10" s="13"/>
     </row>
@@ -17827,16 +17966,16 @@
         <v>55</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="G11" s="27" t="s">
         <v>22</v>
       </c>
       <c r="H11" s="27" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="I11" s="13"/>
     </row>
@@ -17845,19 +17984,19 @@
         <v>17</v>
       </c>
       <c r="D12" s="27" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E12" s="27" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="F12" s="27" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="G12" s="27" t="s">
         <v>35</v>
       </c>
       <c r="H12" s="27" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="I12" s="13"/>
     </row>
@@ -17869,16 +18008,16 @@
         <v>48</v>
       </c>
       <c r="E13" s="27" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="F13" s="27" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="G13" s="27" t="s">
         <v>33</v>
       </c>
       <c r="H13" s="27" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="I13" s="13"/>
     </row>
@@ -17887,13 +18026,13 @@
         <v>17</v>
       </c>
       <c r="D14" s="27" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="E14" s="27" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="F14" s="27" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="G14" s="27" t="s">
         <v>26</v>
@@ -17906,13 +18045,13 @@
         <v>17</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="F15" s="27" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="G15" s="14"/>
       <c r="H15" s="14"/>
@@ -17926,10 +18065,10 @@
         <v>57</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="F16" s="27" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="G16" s="14"/>
       <c r="H16" s="14"/>
@@ -17943,10 +18082,10 @@
         <v>54</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="F17" s="27" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="G17" s="14"/>
       <c r="H17" s="14"/>
@@ -17960,10 +18099,10 @@
         <v>56</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="F18" s="27" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="G18" s="14"/>
       <c r="H18" s="14"/>
@@ -17974,13 +18113,13 @@
         <v>17</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="F19" s="27" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="G19" s="14"/>
       <c r="H19" s="14"/>
@@ -17994,10 +18133,10 @@
         <v>63</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="F20" s="27" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="G20" s="14"/>
       <c r="H20" s="14"/>
@@ -18011,10 +18150,10 @@
         <v>61</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="F21" s="27" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="G21" s="14"/>
       <c r="H21" s="14"/>
@@ -18025,13 +18164,13 @@
         <v>17</v>
       </c>
       <c r="D22" s="27" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="E22" s="27" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="F22" s="27" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="G22" s="14"/>
       <c r="H22" s="14"/>
@@ -18042,13 +18181,13 @@
         <v>17</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="E23" s="27" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="F23" s="27" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="G23" s="14"/>
       <c r="H23" s="14"/>
@@ -18062,10 +18201,10 @@
         <v>58</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="F24" s="27" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="G24" s="14"/>
       <c r="H24" s="14"/>
@@ -18076,13 +18215,13 @@
         <v>17</v>
       </c>
       <c r="D25" s="27" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="E25" s="27" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="F25" s="27" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="G25" s="14"/>
       <c r="H25" s="14"/>
@@ -18096,10 +18235,10 @@
         <v>40</v>
       </c>
       <c r="E26" s="27" t="s">
+        <v>296</v>
+      </c>
+      <c r="F26" s="27" t="s">
         <v>291</v>
-      </c>
-      <c r="F26" s="27" t="s">
-        <v>286</v>
       </c>
       <c r="G26" s="14"/>
       <c r="H26" s="14"/>
@@ -18110,13 +18249,13 @@
         <v>17</v>
       </c>
       <c r="D27" s="27" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="E27" s="27" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="F27" s="27" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="G27" s="14"/>
       <c r="H27" s="14"/>
@@ -18130,10 +18269,10 @@
         <v>50</v>
       </c>
       <c r="E28" s="27" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="F28" s="27" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="G28" s="14"/>
       <c r="H28" s="14"/>
@@ -18144,13 +18283,13 @@
         <v>17</v>
       </c>
       <c r="D29" s="27" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="E29" s="27" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="F29" s="27" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="G29" s="14"/>
       <c r="H29" s="14"/>
@@ -18161,13 +18300,13 @@
         <v>17</v>
       </c>
       <c r="D30" s="27" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="E30" s="27" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="F30" s="27" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="G30" s="14"/>
       <c r="H30" s="14"/>
@@ -18178,13 +18317,13 @@
         <v>17</v>
       </c>
       <c r="D31" s="27" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="E31" s="27" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="F31" s="27" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="G31" s="14"/>
       <c r="H31" s="14"/>
@@ -18198,10 +18337,10 @@
         <v>44</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="F32" s="27" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="G32" s="14"/>
       <c r="H32" s="14"/>
@@ -18212,13 +18351,13 @@
         <v>17</v>
       </c>
       <c r="D33" s="27" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="E33" s="27" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="F33" s="27" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="G33" s="14"/>
       <c r="H33" s="14"/>
@@ -18229,13 +18368,13 @@
         <v>17</v>
       </c>
       <c r="D34" s="27" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="E34" s="27" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="F34" s="27" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="G34" s="14"/>
       <c r="H34" s="14"/>
@@ -18250,7 +18389,7 @@
       </c>
       <c r="E35" s="27"/>
       <c r="F35" s="27" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="G35" s="14"/>
       <c r="H35" s="14"/>
@@ -18265,7 +18404,7 @@
       </c>
       <c r="E36" s="27"/>
       <c r="F36" s="27" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="G36" s="14"/>
       <c r="H36" s="14"/>
@@ -18279,7 +18418,7 @@
         <v>26</v>
       </c>
       <c r="E37" s="27" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="F37" s="27" t="s">
         <v>26</v>
@@ -18296,7 +18435,7 @@
         <v>33</v>
       </c>
       <c r="E38" s="27" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="F38" s="27" t="s">
         <v>33</v>
@@ -18305,14 +18444,16 @@
       <c r="H38" s="14"/>
       <c r="I38" s="13"/>
     </row>
-    <row r="39" spans="3:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="3:9" s="2" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C39" s="29" t="s">
         <v>17</v>
       </c>
       <c r="D39" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="E39" s="27"/>
+      <c r="E39" s="27" t="s">
+        <v>635</v>
+      </c>
       <c r="F39" s="27" t="s">
         <v>35</v>
       </c>
@@ -18373,10 +18514,10 @@
         <v>68</v>
       </c>
       <c r="E43" s="27" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="F43" s="27" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="G43" s="14"/>
       <c r="H43" s="14"/>
@@ -18390,10 +18531,10 @@
         <v>75</v>
       </c>
       <c r="E44" s="27" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="F44" s="27" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="G44" s="14"/>
       <c r="H44" s="14"/>
@@ -18407,7 +18548,7 @@
         <v>78</v>
       </c>
       <c r="E45" s="27" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="F45" s="27" t="s">
         <v>65</v>
@@ -18455,7 +18596,7 @@
       </c>
       <c r="E48" s="27"/>
       <c r="F48" s="27" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="G48" s="14"/>
       <c r="H48" s="14"/>
@@ -18466,11 +18607,11 @@
         <v>64</v>
       </c>
       <c r="D49" s="27" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="E49" s="27"/>
       <c r="F49" s="27" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="G49" s="14"/>
       <c r="H49" s="14"/>
@@ -18484,7 +18625,7 @@
         <v>89</v>
       </c>
       <c r="E50" s="27" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="F50" s="27" t="s">
         <v>65</v>
@@ -18501,7 +18642,7 @@
         <v>92</v>
       </c>
       <c r="E51" s="27" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="F51" s="27" t="s">
         <v>65</v>
@@ -18534,7 +18675,7 @@
       </c>
       <c r="E53" s="27"/>
       <c r="F53" s="27" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="G53" s="14"/>
       <c r="H53" s="14"/>
@@ -18549,7 +18690,7 @@
       </c>
       <c r="E54" s="27"/>
       <c r="F54" s="27" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="G54" s="14"/>
       <c r="H54" s="14"/>
@@ -18564,7 +18705,7 @@
       </c>
       <c r="E55" s="27"/>
       <c r="F55" s="27" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
     </row>
     <row r="56" spans="3:9" ht="144" customHeight="1" x14ac:dyDescent="0.3">
@@ -18575,7 +18716,7 @@
         <v>113</v>
       </c>
       <c r="E56" s="27" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="F56" s="27" t="s">
         <v>65</v>
@@ -18586,13 +18727,13 @@
         <v>17</v>
       </c>
       <c r="D57" s="27" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="E57" s="27" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="F57" s="27" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="58" spans="3:9" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -18603,10 +18744,10 @@
         <v>110</v>
       </c>
       <c r="E58" s="27" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="F58" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="59" spans="3:9" ht="144" customHeight="1" x14ac:dyDescent="0.3">
@@ -18617,10 +18758,10 @@
         <v>132</v>
       </c>
       <c r="E59" s="27" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="F59" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="60" spans="3:9" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -18631,10 +18772,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="27" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="F60" s="27" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="61" spans="3:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -18642,13 +18783,13 @@
         <v>17</v>
       </c>
       <c r="D61" s="27" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="E61" s="27" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="F61" s="27" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
     <row r="62" spans="3:9" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -18659,10 +18800,10 @@
         <v>119</v>
       </c>
       <c r="E62" s="27" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="F62" s="27" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
     </row>
     <row r="63" spans="3:9" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -18670,13 +18811,13 @@
         <v>17</v>
       </c>
       <c r="D63" s="27" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="E63" s="27" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="F63" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="64" spans="3:9" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -18687,7 +18828,7 @@
         <v>122</v>
       </c>
       <c r="E64" s="27" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="F64" s="27" t="s">
         <v>65</v>
@@ -18701,10 +18842,10 @@
         <v>121</v>
       </c>
       <c r="E65" s="27" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="F65" s="27" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="66" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -18715,10 +18856,10 @@
         <v>126</v>
       </c>
       <c r="E66" s="27" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="F66" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="67" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -18726,13 +18867,13 @@
         <v>17</v>
       </c>
       <c r="D67" s="27" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="E67" s="27" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="F67" s="27" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
     </row>
     <row r="68" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -18740,13 +18881,13 @@
         <v>17</v>
       </c>
       <c r="D68" s="27" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="E68" s="27" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="F68" s="27" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="69" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -18757,10 +18898,10 @@
         <v>117</v>
       </c>
       <c r="E69" s="27" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="F69" s="27" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="70" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -18768,13 +18909,13 @@
         <v>17</v>
       </c>
       <c r="D70" s="27" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="E70" s="27" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="F70" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="71" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -18782,13 +18923,13 @@
         <v>17</v>
       </c>
       <c r="D71" s="27" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="E71" s="27" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="F71" s="27" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="72" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -18796,13 +18937,13 @@
         <v>17</v>
       </c>
       <c r="D72" s="27" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="E72" s="27" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="F72" s="27" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="73" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -18813,10 +18954,10 @@
         <v>129</v>
       </c>
       <c r="E73" s="27" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="F73" s="27" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="74" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -18827,10 +18968,10 @@
         <v>130</v>
       </c>
       <c r="E74" s="27" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="F74" s="27" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="75" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -18841,10 +18982,10 @@
         <v>125</v>
       </c>
       <c r="E75" s="27" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="F75" s="27" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="76" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -18855,10 +18996,10 @@
         <v>108</v>
       </c>
       <c r="E76" s="27" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="F76" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="77" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -18869,10 +19010,10 @@
         <v>120</v>
       </c>
       <c r="E77" s="27" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="F77" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="78" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -18883,10 +19024,10 @@
         <v>128</v>
       </c>
       <c r="E78" s="27" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="F78" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="79" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -18897,10 +19038,10 @@
         <v>110</v>
       </c>
       <c r="E79" s="27" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="F79" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="80" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -18911,10 +19052,10 @@
         <v>118</v>
       </c>
       <c r="E80" s="27" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="F80" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="81" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -18925,10 +19066,10 @@
         <v>124</v>
       </c>
       <c r="E81" s="27" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="F81" s="27" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="82" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -18939,7 +19080,7 @@
         <v>111</v>
       </c>
       <c r="E82" s="27" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="F82" s="27" t="s">
         <v>65</v>
@@ -18953,10 +19094,10 @@
         <v>114</v>
       </c>
       <c r="E83" s="27" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F83" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="84" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -18964,13 +19105,13 @@
         <v>17</v>
       </c>
       <c r="D84" s="27" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="E84" s="27" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="F84" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="85" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -18981,10 +19122,10 @@
         <v>131</v>
       </c>
       <c r="E85" s="27" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="F85" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="86" spans="3:6" x14ac:dyDescent="0.3">
@@ -18992,13 +19133,13 @@
         <v>17</v>
       </c>
       <c r="D86" s="27" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="E86" s="27" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="F86" s="27" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="87" spans="3:6" x14ac:dyDescent="0.3">
@@ -19009,10 +19150,10 @@
         <v>123</v>
       </c>
       <c r="E87" s="27" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="F87" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="88" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19023,10 +19164,10 @@
         <v>127</v>
       </c>
       <c r="E88" s="27" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="F88" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="89" spans="3:6" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19037,10 +19178,10 @@
         <v>137</v>
       </c>
       <c r="E89" s="27" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="F89" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="90" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19051,10 +19192,10 @@
         <v>141</v>
       </c>
       <c r="E90" s="27" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="F90" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="91" spans="3:6" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -19065,10 +19206,10 @@
         <v>148</v>
       </c>
       <c r="E91" s="27" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="F91" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="92" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19079,10 +19220,10 @@
         <v>144</v>
       </c>
       <c r="E92" s="27" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="F92" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="93" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19090,13 +19231,13 @@
         <v>17</v>
       </c>
       <c r="D93" s="27" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="E93" s="27" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="F93" s="27" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
     </row>
     <row r="94" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19104,13 +19245,13 @@
         <v>17</v>
       </c>
       <c r="D94" s="27" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="E94" s="27" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="F94" s="27" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
     </row>
     <row r="95" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19121,10 +19262,10 @@
         <v>145</v>
       </c>
       <c r="E95" s="27" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="F95" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="96" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19132,13 +19273,13 @@
         <v>17</v>
       </c>
       <c r="D96" s="27" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="E96" s="27" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="F96" s="27" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
     </row>
     <row r="97" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19146,13 +19287,13 @@
         <v>17</v>
       </c>
       <c r="D97" s="27" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="E97" s="27" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="F97" s="27" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
     </row>
     <row r="98" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -19160,13 +19301,13 @@
         <v>17</v>
       </c>
       <c r="D98" s="27" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="E98" s="27" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="F98" s="27" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
     </row>
     <row r="99" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19174,13 +19315,13 @@
         <v>17</v>
       </c>
       <c r="D99" s="27" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="E99" s="27" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="F99" s="27" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
     </row>
     <row r="100" spans="3:6" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -19188,13 +19329,13 @@
         <v>17</v>
       </c>
       <c r="D100" s="27" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="E100" s="27" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="F100" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="101" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19202,13 +19343,13 @@
         <v>17</v>
       </c>
       <c r="D101" s="27" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="E101" s="27" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="F101" s="27" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
     </row>
     <row r="102" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -19216,13 +19357,13 @@
         <v>17</v>
       </c>
       <c r="D102" s="27" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="E102" s="27" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="F102" s="27" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
     </row>
     <row r="103" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19233,10 +19374,10 @@
         <v>136</v>
       </c>
       <c r="E103" s="27" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="F103" s="27" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
     </row>
     <row r="104" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19247,10 +19388,10 @@
         <v>155</v>
       </c>
       <c r="E104" s="27" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="F104" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="105" spans="3:6" ht="244.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19261,10 +19402,10 @@
         <v>159</v>
       </c>
       <c r="E105" s="27" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="F105" s="27" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
     </row>
     <row r="106" spans="3:6" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19275,10 +19416,10 @@
         <v>163</v>
       </c>
       <c r="E106" s="27" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="F106" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="107" spans="3:6" ht="172.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19286,13 +19427,13 @@
         <v>17</v>
       </c>
       <c r="D107" s="27" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="E107" s="27" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="F107" s="27" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
     </row>
     <row r="108" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19300,13 +19441,13 @@
         <v>17</v>
       </c>
       <c r="D108" s="27" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="E108" s="27" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="F108" s="27" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
     </row>
     <row r="109" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -19314,13 +19455,13 @@
         <v>17</v>
       </c>
       <c r="D109" s="27" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="E109" s="27" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="F109" s="27" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
     </row>
     <row r="110" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19331,10 +19472,10 @@
         <v>165</v>
       </c>
       <c r="E110" s="27" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="F110" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="111" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19342,13 +19483,13 @@
         <v>17</v>
       </c>
       <c r="D111" s="27" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="E111" s="27" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="F111" s="27" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
     </row>
     <row r="112" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -19356,13 +19497,13 @@
         <v>17</v>
       </c>
       <c r="D112" s="27" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="E112" s="27" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="F112" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="113" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19370,13 +19511,13 @@
         <v>17</v>
       </c>
       <c r="D113" s="27" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="E113" s="27" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
       <c r="F113" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="114" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19384,13 +19525,13 @@
         <v>17</v>
       </c>
       <c r="D114" s="27" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="E114" s="27" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="F114" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="115" spans="3:6" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -19401,10 +19542,10 @@
         <v>154</v>
       </c>
       <c r="E115" s="27" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="F115" s="27" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
     </row>
     <row r="116" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19415,10 +19556,10 @@
         <v>167</v>
       </c>
       <c r="E116" s="27" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="F116" s="27" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
     </row>
     <row r="117" spans="3:6" ht="144" customHeight="1" x14ac:dyDescent="0.3">
@@ -19429,10 +19570,10 @@
         <v>151</v>
       </c>
       <c r="E117" s="27" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="F117" s="27" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
     </row>
     <row r="118" spans="3:6" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -19443,10 +19584,10 @@
         <v>135</v>
       </c>
       <c r="E118" s="27" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="F118" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="119" spans="3:6" ht="230.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -19457,10 +19598,10 @@
         <v>142</v>
       </c>
       <c r="E119" s="27" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="F119" s="27" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="120" spans="3:6" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -19471,10 +19612,10 @@
         <v>158</v>
       </c>
       <c r="E120" s="27" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
       <c r="F120" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="121" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19485,10 +19626,10 @@
         <v>139</v>
       </c>
       <c r="E121" s="27" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="F121" s="27" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
     </row>
     <row r="122" spans="3:6" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19499,10 +19640,10 @@
         <v>156</v>
       </c>
       <c r="E122" s="27" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="F122" s="27" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
     </row>
     <row r="123" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19510,13 +19651,13 @@
         <v>17</v>
       </c>
       <c r="D123" s="27" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="E123" s="27" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="F123" s="27" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
     </row>
     <row r="124" spans="3:6" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19527,10 +19668,10 @@
         <v>164</v>
       </c>
       <c r="E124" s="27" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="F124" s="27" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="125" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19541,10 +19682,10 @@
         <v>147</v>
       </c>
       <c r="E125" s="27" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
       <c r="F125" s="27" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
     </row>
     <row r="126" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19555,10 +19696,10 @@
         <v>140</v>
       </c>
       <c r="E126" s="27" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="F126" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="127" spans="3:6" ht="244.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19566,13 +19707,13 @@
         <v>17</v>
       </c>
       <c r="D127" s="27" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="E127" s="27" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="F127" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="128" spans="3:6" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19580,13 +19721,13 @@
         <v>17</v>
       </c>
       <c r="D128" s="27" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="E128" s="27" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="F128" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="129" spans="3:6" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -19594,13 +19735,13 @@
         <v>17</v>
       </c>
       <c r="D129" s="27" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="E129" s="27" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="F129" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="130" spans="3:6" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -19608,13 +19749,13 @@
         <v>17</v>
       </c>
       <c r="D130" s="27" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="E130" s="27" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
       <c r="F130" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="131" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19622,13 +19763,13 @@
         <v>17</v>
       </c>
       <c r="D131" s="27" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
       <c r="E131" s="27" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
       <c r="F131" s="27" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
     </row>
     <row r="132" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -19636,13 +19777,13 @@
         <v>17</v>
       </c>
       <c r="D132" s="27" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="E132" s="27" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="F132" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="133" spans="3:6" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -19650,13 +19791,13 @@
         <v>17</v>
       </c>
       <c r="D133" s="27" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
       <c r="E133" s="27" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="F133" s="27" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="134" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -19664,13 +19805,13 @@
         <v>17</v>
       </c>
       <c r="D134" s="27" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="E134" s="27" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="F134" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="135" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19678,13 +19819,13 @@
         <v>17</v>
       </c>
       <c r="D135" s="27" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="E135" s="27" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="F135" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="136" spans="3:6" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -19692,13 +19833,13 @@
         <v>17</v>
       </c>
       <c r="D136" s="27" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="E136" s="27" t="s">
-        <v>459</v>
+        <v>464</v>
       </c>
       <c r="F136" s="27" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
     </row>
     <row r="137" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19709,10 +19850,10 @@
         <v>138</v>
       </c>
       <c r="E137" s="27" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="F137" s="27" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
     </row>
     <row r="138" spans="3:6" x14ac:dyDescent="0.3">
@@ -19724,7 +19865,7 @@
       </c>
       <c r="E138" s="27"/>
       <c r="F138" s="27" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="139" spans="3:6" x14ac:dyDescent="0.3">
@@ -19736,7 +19877,7 @@
       </c>
       <c r="E139" s="27"/>
       <c r="F139" s="27" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="140" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19747,10 +19888,10 @@
         <v>178</v>
       </c>
       <c r="E140" s="27" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="F140" s="27" t="s">
-        <v>567</v>
+        <v>468</v>
       </c>
     </row>
     <row r="141" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19761,10 +19902,10 @@
         <v>188</v>
       </c>
       <c r="E141" s="27" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="F141" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="142" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -19772,13 +19913,13 @@
         <v>17</v>
       </c>
       <c r="D142" s="27" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="E142" s="27" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="F142" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="143" spans="3:6" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -19789,10 +19930,10 @@
         <v>171</v>
       </c>
       <c r="E143" s="27" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="F143" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="144" spans="3:6" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19803,10 +19944,10 @@
         <v>173</v>
       </c>
       <c r="E144" s="27" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="F144" s="27" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="145" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19817,10 +19958,10 @@
         <v>191</v>
       </c>
       <c r="E145" s="27" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="F145" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="146" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19828,13 +19969,13 @@
         <v>17</v>
       </c>
       <c r="D146" s="27" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="E146" s="27" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="F146" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="147" spans="3:6" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19845,10 +19986,10 @@
         <v>190</v>
       </c>
       <c r="E147" s="27" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="F147" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="148" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19856,13 +19997,13 @@
         <v>17</v>
       </c>
       <c r="D148" s="27" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="E148" s="27" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="F148" s="27" t="s">
-        <v>568</v>
+        <v>480</v>
       </c>
     </row>
     <row r="149" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19870,13 +20011,13 @@
         <v>17</v>
       </c>
       <c r="D149" s="27" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="E149" s="27" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="F149" s="27" t="s">
-        <v>569</v>
+        <v>483</v>
       </c>
     </row>
     <row r="150" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19884,13 +20025,13 @@
         <v>17</v>
       </c>
       <c r="D150" s="27" t="s">
-        <v>476</v>
+        <v>484</v>
       </c>
       <c r="E150" s="27" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="F150" s="27" t="s">
-        <v>570</v>
+        <v>486</v>
       </c>
     </row>
     <row r="151" spans="3:6" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -19901,10 +20042,10 @@
         <v>175</v>
       </c>
       <c r="E151" s="27" t="s">
-        <v>478</v>
+        <v>487</v>
       </c>
       <c r="F151" s="27" t="s">
-        <v>571</v>
+        <v>488</v>
       </c>
     </row>
     <row r="152" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19912,13 +20053,13 @@
         <v>17</v>
       </c>
       <c r="D152" s="27" t="s">
-        <v>479</v>
+        <v>489</v>
       </c>
       <c r="E152" s="27" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="F152" s="27" t="s">
-        <v>570</v>
+        <v>486</v>
       </c>
     </row>
     <row r="153" spans="3:6" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -19929,10 +20070,10 @@
         <v>186</v>
       </c>
       <c r="E153" s="27" t="s">
-        <v>481</v>
+        <v>491</v>
       </c>
       <c r="F153" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="154" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -19940,13 +20081,13 @@
         <v>17</v>
       </c>
       <c r="D154" s="27" t="s">
-        <v>482</v>
+        <v>492</v>
       </c>
       <c r="E154" s="27" t="s">
-        <v>483</v>
+        <v>493</v>
       </c>
       <c r="F154" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="155" spans="3:6" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -19954,13 +20095,13 @@
         <v>17</v>
       </c>
       <c r="D155" s="27" t="s">
-        <v>484</v>
+        <v>494</v>
       </c>
       <c r="E155" s="27" t="s">
-        <v>485</v>
+        <v>495</v>
       </c>
       <c r="F155" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="156" spans="3:6" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -19968,13 +20109,13 @@
         <v>17</v>
       </c>
       <c r="D156" s="27" t="s">
-        <v>486</v>
+        <v>496</v>
       </c>
       <c r="E156" s="27" t="s">
-        <v>487</v>
+        <v>497</v>
       </c>
       <c r="F156" s="27" t="s">
-        <v>568</v>
+        <v>480</v>
       </c>
     </row>
     <row r="157" spans="3:6" x14ac:dyDescent="0.3">
@@ -19986,7 +20127,7 @@
       </c>
       <c r="E157" s="27"/>
       <c r="F157" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="158" spans="3:6" x14ac:dyDescent="0.3">
@@ -19998,7 +20139,7 @@
       </c>
       <c r="E158" s="27"/>
       <c r="F158" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="159" spans="3:6" x14ac:dyDescent="0.3">
@@ -20010,7 +20151,7 @@
       </c>
       <c r="E159" s="27"/>
       <c r="F159" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="160" spans="3:6" x14ac:dyDescent="0.3">
@@ -20022,7 +20163,7 @@
       </c>
       <c r="E160" s="27"/>
       <c r="F160" s="27" t="s">
-        <v>568</v>
+        <v>480</v>
       </c>
     </row>
     <row r="161" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20034,7 +20175,7 @@
       </c>
       <c r="E161" s="27"/>
       <c r="F161" s="27" t="s">
-        <v>570</v>
+        <v>486</v>
       </c>
     </row>
     <row r="162" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20045,10 +20186,10 @@
         <v>192</v>
       </c>
       <c r="E162" s="27" t="s">
-        <v>488</v>
+        <v>498</v>
       </c>
       <c r="F162" s="27" t="s">
-        <v>572</v>
+        <v>499</v>
       </c>
     </row>
     <row r="163" spans="3:6" x14ac:dyDescent="0.3">
@@ -20060,7 +20201,7 @@
       </c>
       <c r="E163" s="27"/>
       <c r="F163" s="27" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="164" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -20068,13 +20209,13 @@
         <v>17</v>
       </c>
       <c r="D164" s="27" t="s">
-        <v>489</v>
+        <v>500</v>
       </c>
       <c r="E164" s="27" t="s">
-        <v>490</v>
+        <v>501</v>
       </c>
       <c r="F164" s="27" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
     </row>
     <row r="165" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -20082,13 +20223,13 @@
         <v>17</v>
       </c>
       <c r="D165" s="27" t="s">
-        <v>492</v>
+        <v>503</v>
       </c>
       <c r="E165" s="27" t="s">
-        <v>493</v>
+        <v>504</v>
       </c>
       <c r="F165" s="27" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
     </row>
     <row r="166" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20096,13 +20237,13 @@
         <v>17</v>
       </c>
       <c r="D166" s="27" t="s">
-        <v>494</v>
+        <v>505</v>
       </c>
       <c r="E166" s="27" t="s">
-        <v>495</v>
+        <v>506</v>
       </c>
       <c r="F166" s="27" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
     </row>
     <row r="167" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20110,13 +20251,13 @@
         <v>17</v>
       </c>
       <c r="D167" s="27" t="s">
-        <v>496</v>
+        <v>507</v>
       </c>
       <c r="E167" s="27" t="s">
-        <v>497</v>
+        <v>508</v>
       </c>
       <c r="F167" s="27" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="168" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20127,10 +20268,10 @@
         <v>204</v>
       </c>
       <c r="E168" s="27" t="s">
-        <v>499</v>
+        <v>510</v>
       </c>
       <c r="F168" s="27" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="169" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20138,13 +20279,13 @@
         <v>17</v>
       </c>
       <c r="D169" s="27" t="s">
-        <v>500</v>
+        <v>511</v>
       </c>
       <c r="E169" s="27" t="s">
-        <v>501</v>
+        <v>512</v>
       </c>
       <c r="F169" s="27" t="s">
-        <v>502</v>
+        <v>513</v>
       </c>
     </row>
     <row r="170" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -20152,13 +20293,13 @@
         <v>17</v>
       </c>
       <c r="D170" s="27" t="s">
-        <v>503</v>
+        <v>514</v>
       </c>
       <c r="E170" s="27" t="s">
-        <v>504</v>
+        <v>515</v>
       </c>
       <c r="F170" s="27" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="171" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -20166,13 +20307,13 @@
         <v>17</v>
       </c>
       <c r="D171" s="27" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E171" s="27" t="s">
-        <v>506</v>
+        <v>517</v>
       </c>
       <c r="F171" s="27" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="172" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20180,13 +20321,13 @@
         <v>17</v>
       </c>
       <c r="D172" s="27" t="s">
-        <v>507</v>
+        <v>518</v>
       </c>
       <c r="E172" s="27" t="s">
-        <v>508</v>
+        <v>519</v>
       </c>
       <c r="F172" s="27" t="s">
-        <v>509</v>
+        <v>520</v>
       </c>
     </row>
     <row r="173" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20197,10 +20338,10 @@
         <v>207</v>
       </c>
       <c r="E173" s="27" t="s">
-        <v>510</v>
+        <v>521</v>
       </c>
       <c r="F173" s="27" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
     </row>
     <row r="174" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -20211,10 +20352,10 @@
         <v>201</v>
       </c>
       <c r="E174" s="27" t="s">
-        <v>512</v>
+        <v>523</v>
       </c>
       <c r="F174" s="27" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
     </row>
     <row r="175" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -20225,10 +20366,10 @@
         <v>205</v>
       </c>
       <c r="E175" s="27" t="s">
-        <v>512</v>
+        <v>523</v>
       </c>
       <c r="F175" s="27" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
     </row>
     <row r="176" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20239,10 +20380,10 @@
         <v>215</v>
       </c>
       <c r="E176" s="27" t="s">
-        <v>513</v>
+        <v>524</v>
       </c>
       <c r="F176" s="27" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
     </row>
     <row r="177" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -20250,13 +20391,13 @@
         <v>17</v>
       </c>
       <c r="D177" s="27" t="s">
-        <v>514</v>
+        <v>525</v>
       </c>
       <c r="E177" s="27" t="s">
-        <v>515</v>
+        <v>526</v>
       </c>
       <c r="F177" s="27" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
     </row>
     <row r="178" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -20267,10 +20408,10 @@
         <v>202</v>
       </c>
       <c r="E178" s="27" t="s">
-        <v>516</v>
+        <v>527</v>
       </c>
       <c r="F178" s="27" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
     </row>
     <row r="179" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -20281,10 +20422,10 @@
         <v>212</v>
       </c>
       <c r="E179" s="27" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="F179" s="27" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="180" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20295,10 +20436,10 @@
         <v>214</v>
       </c>
       <c r="E180" s="27" t="s">
-        <v>518</v>
+        <v>529</v>
       </c>
       <c r="F180" s="27" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="181" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -20309,10 +20450,10 @@
         <v>206</v>
       </c>
       <c r="E181" s="27" t="s">
-        <v>519</v>
+        <v>530</v>
       </c>
       <c r="F181" s="27" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="182" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20323,10 +20464,10 @@
         <v>208</v>
       </c>
       <c r="E182" s="27" t="s">
-        <v>510</v>
+        <v>521</v>
       </c>
       <c r="F182" s="27" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
     </row>
     <row r="183" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20334,13 +20475,13 @@
         <v>17</v>
       </c>
       <c r="D183" s="27" t="s">
-        <v>520</v>
+        <v>531</v>
       </c>
       <c r="E183" s="27" t="s">
-        <v>521</v>
+        <v>532</v>
       </c>
       <c r="F183" s="27" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="184" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -20348,13 +20489,13 @@
         <v>17</v>
       </c>
       <c r="D184" s="27" t="s">
-        <v>522</v>
+        <v>533</v>
       </c>
       <c r="E184" s="27" t="s">
-        <v>523</v>
+        <v>534</v>
       </c>
       <c r="F184" s="27" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="185" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20362,13 +20503,13 @@
         <v>17</v>
       </c>
       <c r="D185" s="27" t="s">
-        <v>524</v>
+        <v>535</v>
       </c>
       <c r="E185" s="27" t="s">
-        <v>525</v>
+        <v>536</v>
       </c>
       <c r="F185" s="27" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
     </row>
     <row r="186" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20376,13 +20517,13 @@
         <v>17</v>
       </c>
       <c r="D186" s="27" t="s">
-        <v>526</v>
+        <v>537</v>
       </c>
       <c r="E186" s="27" t="s">
-        <v>527</v>
+        <v>538</v>
       </c>
       <c r="F186" s="27" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="187" spans="3:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -20390,13 +20531,13 @@
         <v>17</v>
       </c>
       <c r="D187" s="27" t="s">
-        <v>528</v>
+        <v>539</v>
       </c>
       <c r="E187" s="27" t="s">
-        <v>529</v>
+        <v>540</v>
       </c>
       <c r="F187" s="27" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="188" spans="3:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -20404,13 +20545,13 @@
         <v>17</v>
       </c>
       <c r="D188" s="27" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="E188" s="27" t="s">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="F188" s="27" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="189" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20421,10 +20562,10 @@
         <v>210</v>
       </c>
       <c r="E189" s="27" t="s">
-        <v>532</v>
+        <v>543</v>
       </c>
       <c r="F189" s="27" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="190" spans="3:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -20435,125 +20576,277 @@
         <v>213</v>
       </c>
       <c r="E190" s="27" t="s">
-        <v>533</v>
+        <v>544</v>
       </c>
       <c r="F190" s="27" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="191" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C191" s="29"/>
-      <c r="D191" s="27"/>
-      <c r="E191" s="27"/>
-      <c r="F191" s="27"/>
-    </row>
-    <row r="192" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C192" s="29"/>
-      <c r="D192" s="27"/>
-      <c r="E192" s="27"/>
-      <c r="F192" s="27"/>
-    </row>
-    <row r="193" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C193" s="29"/>
-      <c r="D193" s="27"/>
-      <c r="E193" s="27"/>
-      <c r="F193" s="27"/>
-    </row>
-    <row r="194" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C194" s="29"/>
-      <c r="D194" s="27"/>
-      <c r="E194" s="27"/>
-      <c r="F194" s="27"/>
-    </row>
-    <row r="195" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C195" s="29"/>
-      <c r="D195" s="27"/>
-      <c r="E195" s="27"/>
-      <c r="F195" s="27"/>
-    </row>
-    <row r="196" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C196" s="29"/>
-      <c r="D196" s="27"/>
-      <c r="E196" s="27"/>
-      <c r="F196" s="27"/>
-    </row>
-    <row r="197" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C197" s="29"/>
-      <c r="D197" s="27"/>
-      <c r="E197" s="27"/>
-      <c r="F197" s="27"/>
-    </row>
-    <row r="198" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C198" s="29"/>
-      <c r="D198" s="27"/>
-      <c r="E198" s="27"/>
-      <c r="F198" s="27"/>
-    </row>
-    <row r="199" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C199" s="29"/>
-      <c r="D199" s="27"/>
-      <c r="E199" s="27"/>
-      <c r="F199" s="27"/>
-    </row>
-    <row r="200" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C200" s="29"/>
-      <c r="D200" s="27"/>
-      <c r="E200" s="27"/>
-      <c r="F200" s="27"/>
-    </row>
-    <row r="201" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C201" s="29"/>
-      <c r="D201" s="27"/>
-      <c r="E201" s="27"/>
-      <c r="F201" s="27"/>
-    </row>
-    <row r="202" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C202" s="29"/>
-      <c r="D202" s="27"/>
-      <c r="E202" s="27"/>
-      <c r="F202" s="27"/>
-    </row>
-    <row r="203" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C203" s="29"/>
-      <c r="D203" s="27"/>
-      <c r="E203" s="27"/>
-      <c r="F203" s="27"/>
-    </row>
-    <row r="204" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C204" s="29"/>
-      <c r="D204" s="27"/>
-      <c r="E204" s="27"/>
-      <c r="F204" s="27"/>
-    </row>
-    <row r="205" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C205" s="29"/>
-      <c r="D205" s="27"/>
-      <c r="E205" s="27"/>
-      <c r="F205" s="27"/>
-    </row>
-    <row r="206" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C206" s="29"/>
-      <c r="D206" s="27"/>
-      <c r="E206" s="27"/>
-      <c r="F206" s="27"/>
-    </row>
-    <row r="207" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C207" s="29"/>
-      <c r="D207" s="27"/>
-      <c r="E207" s="27"/>
-      <c r="F207" s="27"/>
-    </row>
-    <row r="208" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C208" s="29"/>
-      <c r="D208" s="27"/>
-      <c r="E208" s="27"/>
-      <c r="F208" s="27"/>
-    </row>
-    <row r="209" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C209" s="29"/>
-      <c r="D209" s="27"/>
-      <c r="E209" s="27"/>
-      <c r="F209" s="27"/>
+        <v>444</v>
+      </c>
+    </row>
+    <row r="191" spans="3:6" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="C191" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D191" s="27" t="s">
+        <v>545</v>
+      </c>
+      <c r="E191" s="27" t="s">
+        <v>546</v>
+      </c>
+      <c r="F191" s="27" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="192" spans="3:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C192" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D192" s="27" t="s">
+        <v>548</v>
+      </c>
+      <c r="E192" s="27" t="s">
+        <v>549</v>
+      </c>
+      <c r="F192" s="27" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="193" spans="3:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="C193" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D193" s="27" t="s">
+        <v>551</v>
+      </c>
+      <c r="E193" s="27" t="s">
+        <v>552</v>
+      </c>
+      <c r="F193" s="27" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="194" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C194" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D194" s="27" t="s">
+        <v>554</v>
+      </c>
+      <c r="E194" s="27" t="s">
+        <v>555</v>
+      </c>
+      <c r="F194" s="27" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="195" spans="3:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C195" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D195" s="27" t="s">
+        <v>557</v>
+      </c>
+      <c r="E195" s="27" t="s">
+        <v>558</v>
+      </c>
+      <c r="F195" s="27" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="196" spans="3:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C196" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D196" s="27" t="s">
+        <v>560</v>
+      </c>
+      <c r="E196" s="27" t="s">
+        <v>561</v>
+      </c>
+      <c r="F196" s="27" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="197" spans="3:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="C197" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D197" s="27" t="s">
+        <v>563</v>
+      </c>
+      <c r="E197" s="27" t="s">
+        <v>564</v>
+      </c>
+      <c r="F197" s="27" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="198" spans="3:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C198" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D198" s="27" t="s">
+        <v>566</v>
+      </c>
+      <c r="E198" s="27" t="s">
+        <v>567</v>
+      </c>
+      <c r="F198" s="27" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="199" spans="3:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C199" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D199" s="27" t="s">
+        <v>569</v>
+      </c>
+      <c r="E199" s="27" t="s">
+        <v>570</v>
+      </c>
+      <c r="F199" s="27" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="200" spans="3:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C200" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D200" s="27" t="s">
+        <v>572</v>
+      </c>
+      <c r="E200" s="27" t="s">
+        <v>573</v>
+      </c>
+      <c r="F200" s="27" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="201" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C201" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D201" s="27" t="s">
+        <v>575</v>
+      </c>
+      <c r="E201" s="27" t="s">
+        <v>576</v>
+      </c>
+      <c r="F201" s="27" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="202" spans="3:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C202" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D202" s="27" t="s">
+        <v>578</v>
+      </c>
+      <c r="E202" s="27" t="s">
+        <v>579</v>
+      </c>
+      <c r="F202" s="27" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="203" spans="3:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C203" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D203" s="27" t="s">
+        <v>581</v>
+      </c>
+      <c r="E203" s="27" t="s">
+        <v>582</v>
+      </c>
+      <c r="F203" s="27" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="204" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C204" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D204" s="27" t="s">
+        <v>584</v>
+      </c>
+      <c r="E204" s="27" t="s">
+        <v>585</v>
+      </c>
+      <c r="F204" s="27" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="205" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C205" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D205" s="27" t="s">
+        <v>587</v>
+      </c>
+      <c r="E205" s="27" t="s">
+        <v>588</v>
+      </c>
+      <c r="F205" s="27" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="206" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C206" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D206" s="27" t="s">
+        <v>590</v>
+      </c>
+      <c r="E206" s="27" t="s">
+        <v>591</v>
+      </c>
+      <c r="F206" s="27" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="207" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C207" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D207" s="27" t="s">
+        <v>593</v>
+      </c>
+      <c r="E207" s="27" t="s">
+        <v>594</v>
+      </c>
+      <c r="F207" s="27" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="208" spans="3:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C208" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D208" s="27" t="s">
+        <v>596</v>
+      </c>
+      <c r="E208" s="27" t="s">
+        <v>597</v>
+      </c>
+      <c r="F208" s="27" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="209" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C209" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D209" s="27" t="s">
+        <v>599</v>
+      </c>
+      <c r="E209" s="27" t="s">
+        <v>600</v>
+      </c>
+      <c r="F209" s="27" t="s">
+        <v>601</v>
+      </c>
     </row>
     <row r="210" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C210" s="29"/>
@@ -21276,7 +21569,7 @@
       <c r="F329" s="27"/>
     </row>
   </sheetData>
-  <autoFilter ref="C5:H190" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
+  <autoFilter ref="C5:H209" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -21298,42 +21591,42 @@
   <sheetData>
     <row r="2" spans="2:17" x14ac:dyDescent="0.3">
       <c r="C2" s="2" t="s">
-        <v>534</v>
+        <v>602</v>
       </c>
       <c r="D2" t="s">
-        <v>535</v>
+        <v>603</v>
       </c>
       <c r="G2" t="s">
-        <v>536</v>
+        <v>604</v>
       </c>
       <c r="H2" t="s">
-        <v>537</v>
+        <v>605</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>534</v>
+        <v>602</v>
       </c>
       <c r="J2" t="s">
-        <v>535</v>
+        <v>603</v>
       </c>
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.3">
       <c r="C3" s="2" t="s">
-        <v>538</v>
+        <v>606</v>
       </c>
       <c r="D3" t="s">
-        <v>538</v>
+        <v>606</v>
       </c>
       <c r="E3" t="s">
-        <v>538</v>
+        <v>606</v>
       </c>
       <c r="F3" t="s">
-        <v>539</v>
+        <v>607</v>
       </c>
       <c r="G3" t="s">
-        <v>538</v>
+        <v>606</v>
       </c>
       <c r="I3" t="s">
-        <v>538</v>
+        <v>606</v>
       </c>
     </row>
     <row r="4" spans="2:17" x14ac:dyDescent="0.3">
@@ -21341,19 +21634,19 @@
         <v>7</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>540</v>
+        <v>608</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>541</v>
+        <v>609</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>542</v>
+        <v>610</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>543</v>
+        <v>611</v>
       </c>
       <c r="G4" s="25" t="s">
-        <v>544</v>
+        <v>612</v>
       </c>
     </row>
     <row r="5" spans="2:17" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -21361,61 +21654,61 @@
         <v>24</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>545</v>
+        <v>613</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>546</v>
+        <v>614</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>547</v>
+        <v>615</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>548</v>
+        <v>616</v>
       </c>
       <c r="G5" s="24"/>
       <c r="P5" t="s">
-        <v>549</v>
+        <v>617</v>
       </c>
       <c r="Q5" t="s">
-        <v>550</v>
+        <v>618</v>
       </c>
     </row>
     <row r="6" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B6" s="16"/>
       <c r="C6" s="22" t="s">
-        <v>551</v>
+        <v>619</v>
       </c>
       <c r="D6" s="24"/>
       <c r="E6" s="36" t="s">
-        <v>552</v>
+        <v>620</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>553</v>
+        <v>621</v>
       </c>
       <c r="G6" s="24"/>
       <c r="P6" t="s">
-        <v>554</v>
+        <v>622</v>
       </c>
       <c r="Q6" t="s">
-        <v>555</v>
+        <v>623</v>
       </c>
     </row>
     <row r="7" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B7" s="22"/>
       <c r="C7" s="22" t="s">
-        <v>556</v>
+        <v>624</v>
       </c>
       <c r="D7" s="24"/>
       <c r="E7" s="24"/>
       <c r="F7" s="24" t="s">
-        <v>557</v>
+        <v>625</v>
       </c>
       <c r="G7" s="24"/>
       <c r="P7" t="s">
-        <v>558</v>
+        <v>626</v>
       </c>
       <c r="Q7" t="s">
-        <v>559</v>
+        <v>627</v>
       </c>
     </row>
     <row r="8" spans="2:17" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -21427,16 +21720,16 @@
       <c r="E8" s="24"/>
       <c r="F8" s="24"/>
       <c r="G8" s="24" t="s">
-        <v>560</v>
+        <v>628</v>
       </c>
       <c r="I8" t="s">
-        <v>561</v>
+        <v>629</v>
       </c>
       <c r="P8" t="s">
-        <v>562</v>
+        <v>630</v>
       </c>
       <c r="Q8" t="s">
-        <v>563</v>
+        <v>631</v>
       </c>
     </row>
     <row r="9" spans="2:17" x14ac:dyDescent="0.3">
@@ -21446,10 +21739,10 @@
       <c r="E9" s="24"/>
       <c r="F9" s="24"/>
       <c r="G9" s="24" t="s">
-        <v>564</v>
+        <v>632</v>
       </c>
       <c r="I9" t="s">
-        <v>565</v>
+        <v>633</v>
       </c>
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.3">
@@ -21459,7 +21752,7 @@
       <c r="E10" s="24"/>
       <c r="F10" s="24"/>
       <c r="G10" s="24" t="s">
-        <v>566</v>
+        <v>634</v>
       </c>
     </row>
     <row r="11" spans="2:17" x14ac:dyDescent="0.3">

</xml_diff>